<commit_message>
Added the neural network values
</commit_message>
<xml_diff>
--- a/Results/metrics_all.xlsx
+++ b/Results/metrics_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soham\Documents\soham\codes\logarithmic_multiplier\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF98AF8-4191-4B7A-BBB4-F78C016514A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A26FCE1-8D24-4079-B91D-36C196DE9226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
   <si>
     <t>Active Logic Cells</t>
   </si>
@@ -88,6 +88,51 @@
   </si>
   <si>
     <t>MRED</t>
+  </si>
+  <si>
+    <t>FAST UNIFIED MULTIPLIER NEURAL NETWORK EVALUATION</t>
+  </si>
+  <si>
+    <t>Speed 0</t>
+  </si>
+  <si>
+    <t>Epoch 1/5</t>
+  </si>
+  <si>
+    <t>Epoch 2/5</t>
+  </si>
+  <si>
+    <t>Epoch 3/5</t>
+  </si>
+  <si>
+    <t>Epoch 4/5</t>
+  </si>
+  <si>
+    <t>Epoch 5/5</t>
+  </si>
+  <si>
+    <t>Evaluated in 1000 samles in(s) - (Exact baseline = 3.6s)</t>
+  </si>
+  <si>
+    <t>Baseline = 97.34%</t>
+  </si>
+  <si>
+    <t>Speed 1</t>
+  </si>
+  <si>
+    <t>Evaluated in 1000 samles in(s) - (Exact baseline = 4.0s)</t>
+  </si>
+  <si>
+    <t>Speed 2</t>
+  </si>
+  <si>
+    <t>Evaluated in 1000 samles in(s) - (Exact baseline = 3.8s)</t>
+  </si>
+  <si>
+    <t>Baseline = 97.35%</t>
+  </si>
+  <si>
+    <t>Baseline = 97.37%</t>
   </si>
 </sst>
 </file>
@@ -123,8 +168,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,10 +454,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.1796875" customWidth="1"/>
+    <col min="1" max="1" width="45.08984375" customWidth="1"/>
     <col min="2" max="2" width="12.90625" customWidth="1"/>
     <col min="3" max="3" width="16.26953125" customWidth="1"/>
     <col min="4" max="4" width="12.453125" customWidth="1"/>
@@ -743,7 +792,308 @@
         <v>2.8799999999999999E-2</v>
       </c>
     </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B14">
+        <v>0.2419</v>
+      </c>
+      <c r="C14">
+        <v>0.106</v>
+      </c>
+      <c r="D14">
+        <v>7.6100000000000001E-2</v>
+      </c>
+      <c r="E14">
+        <v>6.0100000000000001E-2</v>
+      </c>
+      <c r="F14">
+        <v>4.6100000000000002E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15">
+        <v>122.7</v>
+      </c>
+      <c r="C15">
+        <v>140.4</v>
+      </c>
+      <c r="D15">
+        <v>121.7</v>
+      </c>
+      <c r="E15">
+        <v>153.9</v>
+      </c>
+      <c r="F15">
+        <v>131</v>
+      </c>
+      <c r="G15">
+        <v>152.5</v>
+      </c>
+      <c r="H15">
+        <v>128.9</v>
+      </c>
+      <c r="I15">
+        <v>146.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.97250000000000003</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0.9728</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.97250000000000003</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.97319999999999995</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.97270000000000001</v>
+      </c>
+      <c r="G16" s="1">
+        <v>0.97330000000000005</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0.97319999999999995</v>
+      </c>
+      <c r="I16" s="1">
+        <v>0.97350000000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B19">
+        <v>0.24529999999999999</v>
+      </c>
+      <c r="C19">
+        <v>0.10249999999999999</v>
+      </c>
+      <c r="D19">
+        <v>7.3099999999999998E-2</v>
+      </c>
+      <c r="E19">
+        <v>5.7200000000000001E-2</v>
+      </c>
+      <c r="F19">
+        <v>4.7199999999999999E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20">
+        <v>131.19999999999999</v>
+      </c>
+      <c r="C20">
+        <v>149</v>
+      </c>
+      <c r="D20">
+        <v>125.7</v>
+      </c>
+      <c r="E20">
+        <v>142.19999999999999</v>
+      </c>
+      <c r="F20">
+        <v>123</v>
+      </c>
+      <c r="G20">
+        <v>141.19999999999999</v>
+      </c>
+      <c r="H20">
+        <v>120.2</v>
+      </c>
+      <c r="I20">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="1">
+        <v>0.97330000000000005</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0.97360000000000002</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0.97330000000000005</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.97370000000000001</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0.97340000000000004</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0.9738</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0.97360000000000002</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0.97370000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B24">
+        <v>0.2417</v>
+      </c>
+      <c r="C24">
+        <v>0.1048</v>
+      </c>
+      <c r="D24">
+        <v>7.4499999999999997E-2</v>
+      </c>
+      <c r="E24">
+        <v>5.6899999999999999E-2</v>
+      </c>
+      <c r="F24">
+        <v>4.65E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25">
+        <v>125.5</v>
+      </c>
+      <c r="C25">
+        <v>145.9</v>
+      </c>
+      <c r="D25">
+        <v>124.1</v>
+      </c>
+      <c r="E25">
+        <v>142.5</v>
+      </c>
+      <c r="F25">
+        <v>120.5</v>
+      </c>
+      <c r="G25">
+        <v>142</v>
+      </c>
+      <c r="H25">
+        <v>141.80000000000001</v>
+      </c>
+      <c r="I25">
+        <v>144.19999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.97289999999999999</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.97399999999999998</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0.9728</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.9738</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0.97299999999999998</v>
+      </c>
+      <c r="G26" s="1">
+        <v>0.97340000000000004</v>
+      </c>
+      <c r="H26" s="1">
+        <v>0.97350000000000003</v>
+      </c>
+      <c r="I26" s="1">
+        <v>0.97389999999999999</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:I12"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Delay and PDP values
</commit_message>
<xml_diff>
--- a/Results/metrics_all.xlsx
+++ b/Results/metrics_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soham\Documents\soham\codes\logarithmic_multiplier\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A26FCE1-8D24-4079-B91D-36C196DE9226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7246C695-69AB-40A4-AD2D-5D365C7069B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Active Logic Cells</t>
   </si>
@@ -133,6 +133,24 @@
   </si>
   <si>
     <t>Baseline = 97.37%</t>
+  </si>
+  <si>
+    <t>Clock period (ns)</t>
+  </si>
+  <si>
+    <t>Worst setup slack (ns)</t>
+  </si>
+  <si>
+    <t>PDP (fJ)</t>
+  </si>
+  <si>
+    <t>Baseline clock frequency (MHz)</t>
+  </si>
+  <si>
+    <t>Maximum operating frquency (MHz)</t>
+  </si>
+  <si>
+    <t>Critical Path Delay (ns)</t>
   </si>
 </sst>
 </file>
@@ -454,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="45.08984375" customWidth="1"/>
@@ -735,7 +753,7 @@
         <v>84.884230370940756</v>
       </c>
       <c r="C10">
-        <f t="shared" ref="C10:I10" si="0">(C6/C7)*100</f>
+        <f t="shared" ref="C10:G10" si="0">(C6/C7)*100</f>
         <v>84.729257985773899</v>
       </c>
       <c r="D10">
@@ -793,306 +811,504 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12">
+        <v>25</v>
+      </c>
+      <c r="C12">
+        <v>25</v>
+      </c>
+      <c r="D12">
+        <v>25</v>
+      </c>
+      <c r="E12">
+        <v>25</v>
+      </c>
+      <c r="F12">
+        <v>25</v>
+      </c>
+      <c r="G12">
+        <v>25</v>
+      </c>
+      <c r="H12">
+        <v>25</v>
+      </c>
+      <c r="I12">
+        <v>25</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" t="s">
-        <v>24</v>
+        <v>34</v>
+      </c>
+      <c r="B13">
+        <v>11.4426063</v>
+      </c>
+      <c r="C13">
+        <v>11.149002039999999</v>
+      </c>
+      <c r="D13">
+        <v>11.282905599999999</v>
+      </c>
+      <c r="E13">
+        <v>11.39517757</v>
+      </c>
+      <c r="F13">
+        <v>10.57641205</v>
+      </c>
+      <c r="G13">
+        <v>9.8150379490000006</v>
+      </c>
+      <c r="H13">
+        <v>10.347497369999999</v>
+      </c>
+      <c r="I13">
+        <v>9.8334632109999998</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
       <c r="B14">
-        <v>0.2419</v>
+        <f>(B12-B13)</f>
+        <v>13.5573937</v>
       </c>
       <c r="C14">
-        <v>0.106</v>
+        <f t="shared" ref="C14:I14" si="1">(C12-C13)</f>
+        <v>13.850997960000001</v>
       </c>
       <c r="D14">
-        <v>7.6100000000000001E-2</v>
+        <f t="shared" si="1"/>
+        <v>13.717094400000001</v>
       </c>
       <c r="E14">
-        <v>6.0100000000000001E-2</v>
+        <f t="shared" si="1"/>
+        <v>13.60482243</v>
       </c>
       <c r="F14">
-        <v>4.6100000000000002E-2</v>
+        <f t="shared" si="1"/>
+        <v>14.42358795</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>15.184962050999999</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>14.652502630000001</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="1"/>
+        <v>15.166536789</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B15">
-        <v>122.7</v>
+        <f>(B2*B14)</f>
+        <v>687.08871271600003</v>
       </c>
       <c r="C15">
-        <v>140.4</v>
+        <f t="shared" ref="C15:I15" si="2">(C2*C14)</f>
+        <v>710.55619534799996</v>
       </c>
       <c r="D15">
-        <v>121.7</v>
+        <f t="shared" si="2"/>
+        <v>758.2809784320001</v>
       </c>
       <c r="E15">
-        <v>153.9</v>
+        <f t="shared" si="2"/>
+        <v>753.70716262200006</v>
       </c>
       <c r="F15">
-        <v>131</v>
+        <f t="shared" si="2"/>
+        <v>910.41687140399995</v>
       </c>
       <c r="G15">
-        <v>152.5</v>
+        <f t="shared" si="2"/>
+        <v>1085.8766362670101</v>
       </c>
       <c r="H15">
-        <v>128.9</v>
+        <f t="shared" si="2"/>
+        <v>1051.0240136499001</v>
       </c>
       <c r="I15">
-        <v>146.4</v>
+        <f t="shared" si="2"/>
+        <v>1176.7715894585101</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="1">
-        <v>0.97250000000000003</v>
-      </c>
-      <c r="C16" s="1">
-        <v>0.9728</v>
-      </c>
-      <c r="D16" s="1">
-        <v>0.97250000000000003</v>
-      </c>
-      <c r="E16" s="1">
-        <v>0.97319999999999995</v>
-      </c>
-      <c r="F16" s="1">
-        <v>0.97270000000000001</v>
-      </c>
-      <c r="G16" s="1">
-        <v>0.97330000000000005</v>
-      </c>
-      <c r="H16" s="1">
-        <v>0.97319999999999995</v>
-      </c>
-      <c r="I16" s="1">
-        <v>0.97350000000000003</v>
+        <v>36</v>
+      </c>
+      <c r="B16">
+        <v>40</v>
+      </c>
+      <c r="C16">
+        <v>40</v>
+      </c>
+      <c r="D16">
+        <v>40</v>
+      </c>
+      <c r="E16">
+        <v>40</v>
+      </c>
+      <c r="F16">
+        <v>40</v>
+      </c>
+      <c r="G16">
+        <v>40</v>
+      </c>
+      <c r="H16">
+        <v>40</v>
+      </c>
+      <c r="I16">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17">
+        <f>1000/(B14)</f>
+        <v>73.760489820399627</v>
+      </c>
+      <c r="C17">
+        <f t="shared" ref="C17:I17" si="3">1000/(C14)</f>
+        <v>72.196963921868914</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="3"/>
+        <v>72.901736391053774</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="3"/>
+        <v>73.503348180046771</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="3"/>
+        <v>69.33087685716923</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="3"/>
+        <v>65.854626217794561</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="3"/>
+        <v>68.247727043745286</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>65.934630556217741</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="A18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>21</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>22</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E19" t="s">
         <v>23</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F19" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B19">
-        <v>0.24529999999999999</v>
-      </c>
-      <c r="C19">
-        <v>0.10249999999999999</v>
-      </c>
-      <c r="D19">
-        <v>7.3099999999999998E-2</v>
-      </c>
-      <c r="E19">
-        <v>5.7200000000000001E-2</v>
-      </c>
-      <c r="F19">
-        <v>4.7199999999999999E-2</v>
-      </c>
-    </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>28</v>
-      </c>
       <c r="B20">
-        <v>131.19999999999999</v>
+        <v>0.2419</v>
       </c>
       <c r="C20">
-        <v>149</v>
+        <v>0.106</v>
       </c>
       <c r="D20">
-        <v>125.7</v>
+        <v>7.6100000000000001E-2</v>
       </c>
       <c r="E20">
-        <v>142.19999999999999</v>
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="F20">
-        <v>123</v>
-      </c>
-      <c r="G20">
-        <v>141.19999999999999</v>
-      </c>
-      <c r="H20">
-        <v>120.2</v>
-      </c>
-      <c r="I20">
-        <v>140</v>
+        <v>4.6100000000000002E-2</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="1">
+        <v>25</v>
+      </c>
+      <c r="B21">
+        <v>122.7</v>
+      </c>
+      <c r="C21">
+        <v>140.4</v>
+      </c>
+      <c r="D21">
+        <v>121.7</v>
+      </c>
+      <c r="E21">
+        <v>153.9</v>
+      </c>
+      <c r="F21">
+        <v>131</v>
+      </c>
+      <c r="G21">
+        <v>152.5</v>
+      </c>
+      <c r="H21">
+        <v>128.9</v>
+      </c>
+      <c r="I21">
+        <v>146.4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="1">
+        <v>0.97250000000000003</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.9728</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.97250000000000003</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.97319999999999995</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0.97270000000000001</v>
+      </c>
+      <c r="G22" s="1">
         <v>0.97330000000000005</v>
       </c>
-      <c r="C21" s="1">
-        <v>0.97360000000000002</v>
-      </c>
-      <c r="D21" s="1">
-        <v>0.97330000000000005</v>
-      </c>
-      <c r="E21" s="1">
-        <v>0.97370000000000001</v>
-      </c>
-      <c r="F21" s="1">
-        <v>0.97340000000000004</v>
-      </c>
-      <c r="G21" s="1">
-        <v>0.9738</v>
-      </c>
-      <c r="H21" s="1">
-        <v>0.97360000000000002</v>
-      </c>
-      <c r="I21" s="1">
-        <v>0.97370000000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>29</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="H22" s="1">
+        <v>0.97319999999999995</v>
+      </c>
+      <c r="I22" s="1">
+        <v>0.97350000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
         <v>20</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C24" t="s">
         <v>21</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D24" t="s">
         <v>22</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E24" t="s">
         <v>23</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B24">
-        <v>0.2417</v>
-      </c>
-      <c r="C24">
-        <v>0.1048</v>
-      </c>
-      <c r="D24">
-        <v>7.4499999999999997E-2</v>
-      </c>
-      <c r="E24">
-        <v>5.6899999999999999E-2</v>
-      </c>
-      <c r="F24">
-        <v>4.65E-2</v>
-      </c>
-    </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>30</v>
-      </c>
       <c r="B25">
-        <v>125.5</v>
+        <v>0.24529999999999999</v>
       </c>
       <c r="C25">
-        <v>145.9</v>
+        <v>0.10249999999999999</v>
       </c>
       <c r="D25">
-        <v>124.1</v>
+        <v>7.3099999999999998E-2</v>
       </c>
       <c r="E25">
-        <v>142.5</v>
+        <v>5.7200000000000001E-2</v>
       </c>
       <c r="F25">
-        <v>120.5</v>
-      </c>
-      <c r="G25">
-        <v>142</v>
-      </c>
-      <c r="H25">
-        <v>141.80000000000001</v>
-      </c>
-      <c r="I25">
-        <v>144.19999999999999</v>
+        <v>4.7199999999999999E-2</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26">
+        <v>131.19999999999999</v>
+      </c>
+      <c r="C26">
+        <v>149</v>
+      </c>
+      <c r="D26">
+        <v>125.7</v>
+      </c>
+      <c r="E26">
+        <v>142.19999999999999</v>
+      </c>
+      <c r="F26">
+        <v>123</v>
+      </c>
+      <c r="G26">
+        <v>141.19999999999999</v>
+      </c>
+      <c r="H26">
+        <v>120.2</v>
+      </c>
+      <c r="I26">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="1">
+        <v>0.97330000000000005</v>
+      </c>
+      <c r="C27" s="1">
+        <v>0.97360000000000002</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.97330000000000005</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.97370000000000001</v>
+      </c>
+      <c r="F27" s="1">
+        <v>0.97340000000000004</v>
+      </c>
+      <c r="G27" s="1">
+        <v>0.9738</v>
+      </c>
+      <c r="H27" s="1">
+        <v>0.97360000000000002</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0.97370000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" t="s">
+        <v>22</v>
+      </c>
+      <c r="E29" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B30">
+        <v>0.2417</v>
+      </c>
+      <c r="C30">
+        <v>0.1048</v>
+      </c>
+      <c r="D30">
+        <v>7.4499999999999997E-2</v>
+      </c>
+      <c r="E30">
+        <v>5.6899999999999999E-2</v>
+      </c>
+      <c r="F30">
+        <v>4.65E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>125.5</v>
+      </c>
+      <c r="C31">
+        <v>145.9</v>
+      </c>
+      <c r="D31">
+        <v>124.1</v>
+      </c>
+      <c r="E31">
+        <v>142.5</v>
+      </c>
+      <c r="F31">
+        <v>120.5</v>
+      </c>
+      <c r="G31">
+        <v>142</v>
+      </c>
+      <c r="H31">
+        <v>141.80000000000001</v>
+      </c>
+      <c r="I31">
+        <v>144.19999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B32" s="1">
         <v>0.97289999999999999</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C32" s="1">
         <v>0.97399999999999998</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D32" s="1">
         <v>0.9728</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E32" s="1">
         <v>0.9738</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F32" s="1">
         <v>0.97299999999999998</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G32" s="1">
         <v>0.97340000000000004</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H32" s="1">
         <v>0.97350000000000003</v>
       </c>
-      <c r="I26" s="1">
+      <c r="I32" s="1">
         <v>0.97389999999999999</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A18:I18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>